<commit_message>
nhap excel co thanh tien trinh, login hien luon kq
</commit_message>
<xml_diff>
--- a/excel/Chitieu2025.xlsx
+++ b/excel/Chitieu2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HK2_NAM_3\Mo_Hinh_Phan_Lop\DO_AN\QuanLyTuyenSinh\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5255DDF3-FB61-4D80-B200-DC3CCE0A8A28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784D21CA-78B1-4705-8A1F-BF8420CDE51C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="447" xr2:uid="{356666A3-8437-8446-8021-A6A0316C3F1D}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t>TT</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>DỰ KIẾN CHỈ TIÊU TUYỂN SINH NĂM 2025</t>
+  </si>
+  <si>
+    <t>Ngưỡng đầu vào</t>
   </si>
 </sst>
 </file>
@@ -369,8 +372,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -705,21 +711,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43024ACF-209E-3E48-A04B-4D5A2F3798A2}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="16.19921875" customWidth="1"/>
     <col min="3" max="3" width="50.69921875" customWidth="1"/>
     <col min="4" max="4" width="10.796875"/>
+    <col min="5" max="5" width="15.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -732,8 +739,11 @@
       <c r="D2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -746,8 +756,11 @@
       <c r="D3">
         <v>40</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -760,8 +773,11 @@
       <c r="D4">
         <v>200</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -774,8 +790,11 @@
       <c r="D5">
         <v>200</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -788,8 +807,11 @@
       <c r="D6">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -802,8 +824,11 @@
       <c r="D7">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -816,8 +841,11 @@
       <c r="D8">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -830,8 +858,11 @@
       <c r="D9">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -844,8 +875,11 @@
       <c r="D10">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -858,8 +892,11 @@
       <c r="D11">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -872,8 +909,11 @@
       <c r="D12">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -886,8 +926,11 @@
       <c r="D13">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -900,8 +943,11 @@
       <c r="D14">
         <v>75</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -914,8 +960,11 @@
       <c r="D15">
         <v>75</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E15">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -928,8 +977,11 @@
       <c r="D16">
         <v>120</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -942,8 +994,11 @@
       <c r="D17">
         <v>60</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -956,8 +1011,11 @@
       <c r="D18">
         <v>40</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -970,8 +1028,11 @@
       <c r="D19">
         <v>253</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -984,8 +1045,11 @@
       <c r="D20">
         <v>100</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -998,8 +1062,11 @@
       <c r="D21">
         <v>30</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -1012,8 +1079,11 @@
       <c r="D22">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -1026,8 +1096,11 @@
       <c r="D23">
         <v>30</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
@@ -1040,8 +1113,11 @@
       <c r="D24">
         <v>80</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E24">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
@@ -1054,8 +1130,11 @@
       <c r="D25">
         <v>140</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
@@ -1068,8 +1147,11 @@
       <c r="D26">
         <v>30</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E26">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -1082,8 +1164,11 @@
       <c r="D27">
         <v>360</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E27">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
@@ -1096,8 +1181,11 @@
       <c r="D28">
         <v>100</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E28">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
@@ -1110,8 +1198,11 @@
       <c r="D29">
         <v>200</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E29">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
@@ -1124,8 +1215,11 @@
       <c r="D30">
         <v>500</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E30">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
@@ -1138,8 +1232,11 @@
       <c r="D31">
         <v>380</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E31">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -1152,8 +1249,11 @@
       <c r="D32">
         <v>50</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E32">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>31</v>
       </c>
@@ -1166,8 +1266,11 @@
       <c r="D33">
         <v>60</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E33">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>32</v>
       </c>
@@ -1180,8 +1283,11 @@
       <c r="D34">
         <v>70</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E34">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>33</v>
       </c>
@@ -1194,8 +1300,11 @@
       <c r="D35">
         <v>210</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
@@ -1208,8 +1317,11 @@
       <c r="D36">
         <v>30</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E36">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>35</v>
       </c>
@@ -1222,8 +1334,11 @@
       <c r="D37">
         <v>80</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E37">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
@@ -1236,8 +1351,11 @@
       <c r="D38">
         <v>90</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E38">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>37</v>
       </c>
@@ -1250,8 +1368,11 @@
       <c r="D39">
         <v>110</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E39">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>38</v>
       </c>
@@ -1264,8 +1385,11 @@
       <c r="D40">
         <v>80</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E40">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>39</v>
       </c>
@@ -1278,8 +1402,11 @@
       <c r="D41">
         <v>400</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E41">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>40</v>
       </c>
@@ -1292,8 +1419,11 @@
       <c r="D42">
         <v>350</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E42">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>41</v>
       </c>
@@ -1306,8 +1436,11 @@
       <c r="D43">
         <v>45</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E43">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>42</v>
       </c>
@@ -1320,8 +1453,11 @@
       <c r="D44">
         <v>45</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E44">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>43</v>
       </c>
@@ -1334,8 +1470,11 @@
       <c r="D45">
         <v>30</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E45">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>44</v>
       </c>
@@ -1348,8 +1487,11 @@
       <c r="D46">
         <v>30</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E46">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1362,8 +1504,11 @@
       <c r="D47">
         <v>90</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E47">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1376,8 +1521,11 @@
       <c r="D48">
         <v>120</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E48">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1389,6 +1537,9 @@
       </c>
       <c r="D49">
         <v>60</v>
+      </c>
+      <c r="E49">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>